<commit_message>
Update CDAP workbook to adjust for proxy reporting
Using CDAP targets from CHTS for people under 18 due to under reporting in BATS
</commit_message>
<xml_diff>
--- a/utilities/calibration/workbook_templates/04_CoordinatedDailyActivityPattern_2023_blank.xlsx
+++ b/utilities/calibration/workbook_templates/04_CoordinatedDailyActivityPattern_2023_blank.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
-  <workbookPr hidePivotFieldList="1"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub\travel-model-one\utilities\calibration\workbook_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{224AA7D1-6253-4440-8332-3EA899DB7DE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF7C2DFD-A6F2-4D6B-8497-E54DE804CF47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="calibration" sheetId="1" r:id="rId1"/>
     <sheet name="modeldata" sheetId="2" r:id="rId2"/>
     <sheet name="BATS 2023" sheetId="3" r:id="rId3"/>
-    <sheet name="TM1 v03 Targets" sheetId="6" r:id="rId4"/>
+    <sheet name="TM1 v03 Targets" sheetId="6" state="hidden" r:id="rId4"/>
     <sheet name="PersonType Chart" sheetId="5" r:id="rId5"/>
   </sheets>
   <externalReferences>
@@ -31,7 +31,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId7"/>
+    <pivotCache cacheId="6" r:id="rId7"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -53,6 +53,30 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Melody Tsao</author>
+  </authors>
+  <commentList>
+    <comment ref="D18" authorId="0" shapeId="0" xr:uid="{1D46B84C-B797-4451-A092-8EBD1927B57D}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">CHTS Targets from 1.5.2 Calibration Workbook
+</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>PBS&amp;J Employee</author>
@@ -111,7 +135,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="50">
   <si>
     <t>H</t>
   </si>
@@ -259,6 +283,9 @@
   <si>
     <t>Source: M:/Development/Travel Model One/Calibration/Version 1.7/2023_BATS_Summaries/pipeline_mt_20260821_NoMon_rmo/ctramp_2023/BATS_Summaries/dap_summaries.csv</t>
   </si>
+  <si>
+    <t>**BATS 2023 was under-reporting mandatory tours for students under 18, most likely due to proxy reporting. As a result, we will not be using BATS CDAP share for students under 18 and keep the targets from the previous calibration (CHTS)</t>
+  </si>
 </sst>
 </file>
 
@@ -270,7 +297,7 @@
     <numFmt numFmtId="166" formatCode="0.0000;[Red]\-0.0000"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -379,6 +406,18 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -501,7 +540,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -597,15 +636,16 @@
     <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="5" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1980,7 +2020,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="8668550" cy="6291303"/>
+    <xdr:ext cx="8677362" cy="6300482"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
@@ -2293,7 +2333,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{425DF6BC-449A-4A16-B9F3-1C22AC562EC2}" name="PivotTable5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{425DF6BC-449A-4A16-B9F3-1C22AC562EC2}" name="PivotTable5" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="I5:M15" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField axis="axisRow" showAll="0">
@@ -5648,19 +5688,20 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor theme="8"/>
   </sheetPr>
-  <dimension ref="B1:M77"/>
+  <dimension ref="B1:M79"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.5703125" customWidth="1"/>
     <col min="8" max="8" width="24.140625" customWidth="1"/>
-    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="12" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="10" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10" bestFit="1" customWidth="1"/>
     <col min="15" max="17" width="7.42578125" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="10" bestFit="1" customWidth="1"/>
   </cols>
@@ -6011,7 +6052,7 @@
       <c r="C16" t="s">
         <v>1</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="74">
         <v>5095.9923076611367</v>
       </c>
     </row>
@@ -6022,174 +6063,172 @@
       <c r="C17" t="s">
         <v>2</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="74">
         <v>562978.37455945229</v>
       </c>
       <c r="E17" s="2"/>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B18">
+      <c r="B18" s="70">
         <v>6</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="70" t="s">
         <v>0</v>
       </c>
       <c r="D18" s="2">
+        <v>17630.20679</v>
+      </c>
+      <c r="E18" s="2">
         <v>41115.091661171064</v>
       </c>
-      <c r="E18" s="2"/>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B19">
+      <c r="B19" s="70">
         <v>6</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="70" t="s">
         <v>1</v>
       </c>
       <c r="D19" s="2">
+        <v>123094.58867</v>
+      </c>
+      <c r="E19" s="2">
         <v>32780.663158173164</v>
       </c>
-      <c r="E19" s="2"/>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B20">
+      <c r="B20" s="70">
         <v>6</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="70" t="s">
         <v>2</v>
       </c>
       <c r="D20" s="2">
+        <v>17712.811699999998</v>
+      </c>
+      <c r="E20" s="2">
         <v>41918.179611378931</v>
       </c>
-      <c r="E20" s="2"/>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B21">
+      <c r="B21" s="70">
         <v>7</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="70" t="s">
         <v>0</v>
       </c>
       <c r="D21" s="2">
+        <v>85466.730259999997</v>
+      </c>
+      <c r="E21" s="2">
         <v>247900.7678317161</v>
       </c>
-      <c r="E21" s="2"/>
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B22">
+      <c r="B22" s="70">
         <v>7</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="70" t="s">
         <v>1</v>
       </c>
       <c r="D22" s="2">
+        <v>665066.56470999995</v>
+      </c>
+      <c r="E22" s="2">
         <v>140853.46659383521</v>
       </c>
-      <c r="E22" s="2"/>
     </row>
     <row r="23" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B23">
+      <c r="B23" s="70">
         <v>7</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="70" t="s">
         <v>2</v>
       </c>
       <c r="D23" s="2">
+        <v>64858.529419999999</v>
+      </c>
+      <c r="E23" s="2">
         <v>140850.42326779067</v>
       </c>
-      <c r="E23" s="2"/>
     </row>
     <row r="24" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B24">
+      <c r="B24" s="70">
         <v>8</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="70" t="s">
         <v>0</v>
       </c>
       <c r="D24" s="2">
+        <v>121625.49533999999</v>
+      </c>
+      <c r="E24" s="2">
         <v>157345.89475843927</v>
       </c>
-      <c r="E24" s="2"/>
     </row>
     <row r="25" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B25" s="70">
         <v>8</v>
       </c>
-      <c r="C25" t="s">
-        <v>1</v>
-      </c>
-      <c r="D25">
+      <c r="C25" s="70" t="s">
+        <v>1</v>
+      </c>
+      <c r="D25" s="2">
+        <v>138048.92214000001</v>
+      </c>
+      <c r="E25" s="70">
         <v>64377.458058831013</v>
       </c>
-      <c r="E25" s="2"/>
     </row>
     <row r="26" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B26">
+      <c r="B26" s="70">
         <v>8</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="70" t="s">
         <v>2</v>
       </c>
-      <c r="D26">
+      <c r="D26" s="2">
+        <v>145623.69245999999</v>
+      </c>
+      <c r="E26" s="70">
         <v>39919.065974013021</v>
       </c>
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B27" s="2" t="s">
+      <c r="B27" s="70" t="s">
+        <v>49</v>
+      </c>
+      <c r="C27" s="70"/>
+      <c r="D27" s="70"/>
+    </row>
+    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B29" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C27" s="1"/>
-      <c r="D27" s="1"/>
-      <c r="E27" s="1"/>
-    </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B28" s="1" t="s">
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+    </row>
+    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B30" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
-      <c r="E28" s="1"/>
-    </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B29" s="1" t="s">
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+    </row>
+    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B31" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C29" s="1" t="s">
+      <c r="C31" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D29" s="1" t="s">
+      <c r="D31" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E29" s="1" t="s">
+      <c r="E31" s="1" t="s">
         <v>43</v>
-      </c>
-    </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B30">
-        <v>1</v>
-      </c>
-      <c r="C30" t="s">
-        <v>0</v>
-      </c>
-      <c r="D30">
-        <v>20972.980538993601</v>
-      </c>
-      <c r="E30">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B31">
-        <v>1</v>
-      </c>
-      <c r="C31" t="s">
-        <v>1</v>
-      </c>
-      <c r="D31">
-        <v>101791.443381039</v>
-      </c>
-      <c r="E31">
-        <v>410</v>
       </c>
     </row>
     <row r="32" spans="2:5" x14ac:dyDescent="0.25">
@@ -6197,41 +6236,41 @@
         <v>1</v>
       </c>
       <c r="C32" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D32">
-        <v>56525.7782478925</v>
+        <v>20972.980538993601</v>
       </c>
       <c r="E32">
-        <v>265</v>
+        <v>145</v>
       </c>
     </row>
     <row r="33" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B33">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C33" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D33">
-        <v>9363.2104923139996</v>
+        <v>101791.443381039</v>
       </c>
       <c r="E33">
-        <v>31</v>
+        <v>410</v>
       </c>
     </row>
     <row r="34" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B34">
+        <v>1</v>
+      </c>
+      <c r="C34" t="s">
         <v>2</v>
       </c>
-      <c r="C34" t="s">
-        <v>1</v>
-      </c>
       <c r="D34">
-        <v>29187.200693063402</v>
+        <v>56525.7782478925</v>
       </c>
       <c r="E34">
-        <v>58</v>
+        <v>265</v>
       </c>
     </row>
     <row r="35" spans="2:5" x14ac:dyDescent="0.25">
@@ -6239,41 +6278,41 @@
         <v>2</v>
       </c>
       <c r="C35" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D35">
-        <v>28107.324162689001</v>
+        <v>9363.2104923139996</v>
       </c>
       <c r="E35">
-        <v>84</v>
+        <v>31</v>
       </c>
     </row>
     <row r="36" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B36">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C36" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D36">
-        <v>2587.17097574738</v>
+        <v>29187.200693063402</v>
       </c>
       <c r="E36">
-        <v>8</v>
+        <v>58</v>
       </c>
     </row>
     <row r="37" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B37">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C37" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D37">
-        <v>5272.2016418558496</v>
+        <v>28107.324162689001</v>
       </c>
       <c r="E37">
-        <v>22</v>
+        <v>84</v>
       </c>
     </row>
     <row r="38" spans="2:5" x14ac:dyDescent="0.25">
@@ -6281,97 +6320,97 @@
         <v>3</v>
       </c>
       <c r="C38" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D38">
-        <v>14187.895576548101</v>
+        <v>2587.17097574738</v>
       </c>
       <c r="E38">
-        <v>45</v>
+        <v>8</v>
       </c>
     </row>
     <row r="39" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B39">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C39" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D39">
-        <v>10909.387874141699</v>
+        <v>5272.2016418558496</v>
       </c>
       <c r="E39">
-        <v>55</v>
+        <v>22</v>
       </c>
     </row>
     <row r="40" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B40">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C40" t="s">
         <v>2</v>
       </c>
       <c r="D40">
-        <v>38765.573310295011</v>
+        <v>14187.895576548101</v>
       </c>
       <c r="E40">
-        <v>140</v>
+        <v>45</v>
       </c>
     </row>
     <row r="41" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B41">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C41" t="s">
         <v>0</v>
       </c>
       <c r="D41">
-        <v>34940.3033849606</v>
+        <v>10909.387874141699</v>
       </c>
       <c r="E41">
-        <v>110</v>
+        <v>55</v>
       </c>
     </row>
     <row r="42" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B42">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C42" t="s">
         <v>2</v>
       </c>
       <c r="D42">
-        <v>52565.235958389538</v>
+        <v>38765.573310295011</v>
       </c>
       <c r="E42">
-        <v>262</v>
+        <v>140</v>
       </c>
     </row>
     <row r="43" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B43">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C43" t="s">
         <v>0</v>
       </c>
       <c r="D43">
-        <v>3795.8709036518198</v>
+        <v>34940.3033849606</v>
       </c>
       <c r="E43">
-        <v>5</v>
+        <v>110</v>
       </c>
     </row>
     <row r="44" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B44">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C44" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D44">
-        <v>6531.0686161737603</v>
+        <v>52565.235958389538</v>
       </c>
       <c r="E44">
-        <v>4</v>
+        <v>262</v>
       </c>
     </row>
     <row r="45" spans="2:5" x14ac:dyDescent="0.25">
@@ -6379,41 +6418,41 @@
         <v>6</v>
       </c>
       <c r="C45" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D45">
-        <v>4233.5977867305201</v>
+        <v>3795.8709036518198</v>
       </c>
       <c r="E45">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="46" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B46">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C46" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D46">
-        <v>31643.1944620621</v>
+        <v>6531.0686161737603</v>
       </c>
       <c r="E46">
-        <v>38</v>
+        <v>4</v>
       </c>
     </row>
     <row r="47" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B47">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C47" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D47">
-        <v>14117.8259404212</v>
+        <v>4233.5977867305201</v>
       </c>
       <c r="E47">
-        <v>13</v>
+        <v>3</v>
       </c>
     </row>
     <row r="48" spans="2:5" x14ac:dyDescent="0.25">
@@ -6421,41 +6460,41 @@
         <v>7</v>
       </c>
       <c r="C48" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D48">
-        <v>16081.6986499751</v>
+        <v>31643.1944620621</v>
       </c>
       <c r="E48">
-        <v>15</v>
+        <v>38</v>
       </c>
     </row>
     <row r="49" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B49">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C49" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D49">
-        <v>20577.984808375099</v>
+        <v>14117.8259404212</v>
       </c>
       <c r="E49">
-        <v>22</v>
+        <v>13</v>
       </c>
     </row>
     <row r="50" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B50">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C50" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D50">
-        <v>8248.9312060110606</v>
+        <v>16081.6986499751</v>
       </c>
       <c r="E50">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="51" spans="2:5" x14ac:dyDescent="0.25">
@@ -6463,65 +6502,65 @@
         <v>8</v>
       </c>
       <c r="C51" t="s">
+        <v>0</v>
+      </c>
+      <c r="D51">
+        <v>20577.984808375099</v>
+      </c>
+      <c r="E51">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="52" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B52">
+        <v>8</v>
+      </c>
+      <c r="C52" t="s">
+        <v>1</v>
+      </c>
+      <c r="D52">
+        <v>8248.9312060110606</v>
+      </c>
+      <c r="E52">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="53" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B53">
+        <v>8</v>
+      </c>
+      <c r="C53" t="s">
         <v>2</v>
       </c>
-      <c r="D51">
+      <c r="D53">
         <v>4558.7508507235698</v>
       </c>
-      <c r="E51">
+      <c r="E53">
         <v>4</v>
       </c>
     </row>
-    <row r="53" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B53" s="2" t="s">
+    <row r="55" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B55" s="2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="54" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B54" s="1" t="s">
+    <row r="56" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B56" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="55" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B55" t="s">
+    <row r="57" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B57" t="s">
         <v>40</v>
       </c>
-      <c r="C55" t="s">
+      <c r="C57" t="s">
         <v>41</v>
       </c>
-      <c r="D55" t="s">
+      <c r="D57" t="s">
         <v>42</v>
       </c>
-      <c r="E55" t="s">
+      <c r="E57" t="s">
         <v>43</v>
-      </c>
-    </row>
-    <row r="56" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B56">
-        <v>1</v>
-      </c>
-      <c r="C56" t="s">
-        <v>0</v>
-      </c>
-      <c r="D56">
-        <v>63549.153434615902</v>
-      </c>
-      <c r="E56">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="57" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B57">
-        <v>1</v>
-      </c>
-      <c r="C57" t="s">
-        <v>1</v>
-      </c>
-      <c r="D57">
-        <v>210535.026176057</v>
-      </c>
-      <c r="E57">
-        <v>671</v>
       </c>
     </row>
     <row r="58" spans="2:5" x14ac:dyDescent="0.25">
@@ -6529,41 +6568,41 @@
         <v>1</v>
       </c>
       <c r="C58" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D58">
-        <v>121351.542268502</v>
+        <v>63549.153434615902</v>
       </c>
       <c r="E58">
-        <v>416</v>
+        <v>268</v>
       </c>
     </row>
     <row r="59" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B59">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C59" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D59">
-        <v>20968.7890230091</v>
+        <v>210535.026176057</v>
       </c>
       <c r="E59">
-        <v>49</v>
+        <v>671</v>
       </c>
     </row>
     <row r="60" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
         <v>2</v>
       </c>
-      <c r="C60" t="s">
-        <v>1</v>
-      </c>
       <c r="D60">
-        <v>62137.604970189903</v>
+        <v>121351.542268502</v>
       </c>
       <c r="E60">
-        <v>92</v>
+        <v>416</v>
       </c>
     </row>
     <row r="61" spans="2:5" x14ac:dyDescent="0.25">
@@ -6571,41 +6610,41 @@
         <v>2</v>
       </c>
       <c r="C61" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D61">
-        <v>56617.428037848404</v>
+        <v>20968.7890230091</v>
       </c>
       <c r="E61">
-        <v>133</v>
+        <v>49</v>
       </c>
     </row>
     <row r="62" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B62">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C62" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D62">
-        <v>4916.5079167325503</v>
+        <v>62137.604970189903</v>
       </c>
       <c r="E62">
-        <v>19</v>
+        <v>92</v>
       </c>
     </row>
     <row r="63" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B63">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C63" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D63">
-        <v>11219.7352089292</v>
+        <v>56617.428037848404</v>
       </c>
       <c r="E63">
-        <v>33</v>
+        <v>133</v>
       </c>
     </row>
     <row r="64" spans="2:5" x14ac:dyDescent="0.25">
@@ -6613,97 +6652,97 @@
         <v>3</v>
       </c>
       <c r="C64" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D64">
-        <v>30372.661147028601</v>
+        <v>4916.5079167325503</v>
       </c>
       <c r="E64">
-        <v>77</v>
+        <v>19</v>
       </c>
     </row>
     <row r="65" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B65">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C65" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D65">
-        <v>33377.814186217001</v>
+        <v>11219.7352089292</v>
       </c>
       <c r="E65">
-        <v>100</v>
+        <v>33</v>
       </c>
     </row>
     <row r="66" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B66">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C66" t="s">
         <v>2</v>
       </c>
       <c r="D66">
-        <v>70367.585458441914</v>
+        <v>30372.661147028601</v>
       </c>
       <c r="E66">
-        <v>202</v>
+        <v>77</v>
       </c>
     </row>
     <row r="67" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B67">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C67" t="s">
         <v>0</v>
       </c>
       <c r="D67">
-        <v>69883.099397594095</v>
+        <v>33377.814186217001</v>
       </c>
       <c r="E67">
-        <v>202</v>
+        <v>100</v>
       </c>
     </row>
     <row r="68" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B68">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C68" t="s">
         <v>2</v>
       </c>
       <c r="D68">
-        <v>132239.30044086539</v>
+        <v>70367.585458441914</v>
       </c>
       <c r="E68">
-        <v>513</v>
+        <v>202</v>
       </c>
     </row>
     <row r="69" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B69">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C69" t="s">
         <v>0</v>
       </c>
       <c r="D69">
-        <v>7719.92068896827</v>
+        <v>69883.099397594095</v>
       </c>
       <c r="E69">
-        <v>10</v>
+        <v>202</v>
       </c>
     </row>
     <row r="70" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B70">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C70" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D70">
-        <v>6670.6837531622796</v>
+        <v>132239.30044086539</v>
       </c>
       <c r="E70">
-        <v>5</v>
+        <v>513</v>
       </c>
     </row>
     <row r="71" spans="2:5" x14ac:dyDescent="0.25">
@@ -6711,41 +6750,41 @@
         <v>6</v>
       </c>
       <c r="C71" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D71">
-        <v>4233.5977867305201</v>
+        <v>7719.92068896827</v>
       </c>
       <c r="E71">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="72" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B72">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C72" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D72">
-        <v>47157.520468889401</v>
+        <v>6670.6837531622796</v>
       </c>
       <c r="E72">
-        <v>51</v>
+        <v>5</v>
       </c>
     </row>
     <row r="73" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B73">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C73" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D73">
-        <v>27508.592579624699</v>
+        <v>4233.5977867305201</v>
       </c>
       <c r="E73">
-        <v>25</v>
+        <v>3</v>
       </c>
     </row>
     <row r="74" spans="2:5" x14ac:dyDescent="0.25">
@@ -6753,41 +6792,41 @@
         <v>7</v>
       </c>
       <c r="C74" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D74">
-        <v>26449.980666032399</v>
+        <v>47157.520468889401</v>
       </c>
       <c r="E74">
-        <v>24</v>
+        <v>51</v>
       </c>
     </row>
     <row r="75" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B75">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C75" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D75">
-        <v>31749.7412333293</v>
+        <v>27508.592579624699</v>
       </c>
       <c r="E75">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="76" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B76">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C76" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D76">
-        <v>13066.8121666193</v>
+        <v>26449.980666032399</v>
       </c>
       <c r="E76">
-        <v>12</v>
+        <v>24</v>
       </c>
     </row>
     <row r="77" spans="2:5" x14ac:dyDescent="0.25">
@@ -6795,17 +6834,46 @@
         <v>8</v>
       </c>
       <c r="C77" t="s">
+        <v>0</v>
+      </c>
+      <c r="D77">
+        <v>31749.7412333293</v>
+      </c>
+      <c r="E77">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="78" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B78">
+        <v>8</v>
+      </c>
+      <c r="C78" t="s">
+        <v>1</v>
+      </c>
+      <c r="D78">
+        <v>13066.8121666193</v>
+      </c>
+      <c r="E78">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="79" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B79">
+        <v>8</v>
+      </c>
+      <c r="C79" t="s">
         <v>2</v>
       </c>
-      <c r="D77">
+      <c r="D79">
         <v>11381.3647679572</v>
       </c>
-      <c r="E77">
+      <c r="E79">
         <v>7</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -6831,19 +6899,19 @@
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" s="72" t="s">
+      <c r="A2" s="73" t="s">
         <v>35</v>
       </c>
-      <c r="B2" s="72"/>
-      <c r="C2" s="72"/>
-      <c r="D2" s="72"/>
-      <c r="E2" s="72"/>
+      <c r="B2" s="73"/>
+      <c r="C2" s="73"/>
+      <c r="D2" s="73"/>
+      <c r="E2" s="73"/>
       <c r="F2" s="60"/>
-      <c r="H2" s="73"/>
-      <c r="I2" s="73"/>
-      <c r="J2" s="73"/>
-      <c r="K2" s="73"/>
-      <c r="L2" s="73"/>
+      <c r="H2" s="71"/>
+      <c r="I2" s="71"/>
+      <c r="J2" s="71"/>
+      <c r="K2" s="71"/>
+      <c r="L2" s="71"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="50" t="s">
@@ -7112,19 +7180,19 @@
       <c r="F13" s="50"/>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A14" s="72" t="s">
+      <c r="A14" s="73" t="s">
         <v>34</v>
       </c>
-      <c r="B14" s="72"/>
-      <c r="C14" s="72"/>
-      <c r="D14" s="72"/>
-      <c r="E14" s="72"/>
+      <c r="B14" s="73"/>
+      <c r="C14" s="73"/>
+      <c r="D14" s="73"/>
+      <c r="E14" s="73"/>
       <c r="F14" s="60"/>
-      <c r="H14" s="73"/>
-      <c r="I14" s="73"/>
-      <c r="J14" s="73"/>
-      <c r="K14" s="73"/>
-      <c r="L14" s="73"/>
+      <c r="H14" s="71"/>
+      <c r="I14" s="71"/>
+      <c r="J14" s="71"/>
+      <c r="K14" s="71"/>
+      <c r="L14" s="71"/>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="50" t="s">
@@ -7386,19 +7454,19 @@
       <c r="A25" s="57"/>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A27" s="73" t="s">
+      <c r="A27" s="71" t="s">
         <v>33</v>
       </c>
-      <c r="B27" s="73"/>
-      <c r="C27" s="73"/>
-      <c r="D27" s="73"/>
-      <c r="E27" s="73"/>
+      <c r="B27" s="71"/>
+      <c r="C27" s="71"/>
+      <c r="D27" s="71"/>
+      <c r="E27" s="71"/>
       <c r="F27" s="56"/>
-      <c r="H27" s="73"/>
-      <c r="I27" s="73"/>
-      <c r="J27" s="73"/>
-      <c r="K27" s="73"/>
-      <c r="L27" s="73"/>
+      <c r="H27" s="71"/>
+      <c r="I27" s="71"/>
+      <c r="J27" s="71"/>
+      <c r="K27" s="71"/>
+      <c r="L27" s="71"/>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="46" t="s">
@@ -7428,20 +7496,20 @@
       <c r="A29" s="46" t="s">
         <v>7</v>
       </c>
-      <c r="B29" s="71">
+      <c r="B29" s="72">
         <v>0.79</v>
       </c>
-      <c r="C29" s="71">
+      <c r="C29" s="72">
         <v>0.12</v>
       </c>
-      <c r="D29" s="71">
+      <c r="D29" s="72">
         <v>0.09</v>
       </c>
-      <c r="E29" s="71">
+      <c r="E29" s="72">
         <f>SUM(B29:D29)</f>
         <v>1</v>
       </c>
-      <c r="F29" s="71">
+      <c r="F29" s="72">
         <v>0.47599999999999998</v>
       </c>
       <c r="I29" s="64"/>
@@ -7453,11 +7521,11 @@
       <c r="A30" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="B30" s="71"/>
-      <c r="C30" s="71"/>
-      <c r="D30" s="71"/>
-      <c r="E30" s="71"/>
-      <c r="F30" s="71"/>
+      <c r="B30" s="72"/>
+      <c r="C30" s="72"/>
+      <c r="D30" s="72"/>
+      <c r="E30" s="72"/>
+      <c r="F30" s="72"/>
       <c r="I30" s="64"/>
       <c r="J30" s="64"/>
       <c r="K30" s="64"/>
@@ -7492,20 +7560,20 @@
       <c r="A32" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="71">
-        <v>0</v>
-      </c>
-      <c r="C32" s="71">
+      <c r="B32" s="72">
+        <v>0</v>
+      </c>
+      <c r="C32" s="72">
         <v>0.8</v>
       </c>
-      <c r="D32" s="71">
+      <c r="D32" s="72">
         <v>0.2</v>
       </c>
-      <c r="E32" s="71">
+      <c r="E32" s="72">
         <f>SUM(B32:D32)</f>
         <v>1</v>
       </c>
-      <c r="F32" s="71">
+      <c r="F32" s="72">
         <v>0.22600000000000001</v>
       </c>
       <c r="I32" s="64"/>
@@ -7517,11 +7585,11 @@
       <c r="A33" s="46" t="s">
         <v>11</v>
       </c>
-      <c r="B33" s="71"/>
-      <c r="C33" s="71"/>
-      <c r="D33" s="71"/>
-      <c r="E33" s="71"/>
-      <c r="F33" s="71"/>
+      <c r="B33" s="72"/>
+      <c r="C33" s="72"/>
+      <c r="D33" s="72"/>
+      <c r="E33" s="72"/>
+      <c r="F33" s="72"/>
       <c r="I33" s="64"/>
       <c r="J33" s="64"/>
       <c r="K33" s="64"/>
@@ -7531,20 +7599,20 @@
       <c r="A34" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="B34" s="71">
+      <c r="B34" s="72">
         <v>0.65</v>
       </c>
-      <c r="C34" s="71">
+      <c r="C34" s="72">
         <v>0.2</v>
       </c>
-      <c r="D34" s="71">
+      <c r="D34" s="72">
         <v>0.15</v>
       </c>
-      <c r="E34" s="71">
+      <c r="E34" s="72">
         <f>SUM(B34:D34)</f>
         <v>1</v>
       </c>
-      <c r="F34" s="71">
+      <c r="F34" s="72">
         <v>0.246</v>
       </c>
       <c r="I34" s="64"/>
@@ -7556,11 +7624,11 @@
       <c r="A35" s="46" t="s">
         <v>13</v>
       </c>
-      <c r="B35" s="71"/>
-      <c r="C35" s="71"/>
-      <c r="D35" s="71"/>
-      <c r="E35" s="71"/>
-      <c r="F35" s="71"/>
+      <c r="B35" s="72"/>
+      <c r="C35" s="72"/>
+      <c r="D35" s="72"/>
+      <c r="E35" s="72"/>
+      <c r="F35" s="72"/>
       <c r="I35" s="64"/>
       <c r="J35" s="64"/>
       <c r="K35" s="64"/>
@@ -7570,11 +7638,11 @@
       <c r="A36" s="46" t="s">
         <v>14</v>
       </c>
-      <c r="B36" s="71"/>
-      <c r="C36" s="71"/>
-      <c r="D36" s="71"/>
-      <c r="E36" s="71"/>
-      <c r="F36" s="71"/>
+      <c r="B36" s="72"/>
+      <c r="C36" s="72"/>
+      <c r="D36" s="72"/>
+      <c r="E36" s="72"/>
+      <c r="F36" s="72"/>
       <c r="I36" s="64"/>
       <c r="J36" s="64"/>
       <c r="K36" s="64"/>
@@ -7634,11 +7702,11 @@
       <c r="F40" s="54" t="s">
         <v>32</v>
       </c>
-      <c r="H40" s="73"/>
-      <c r="I40" s="73"/>
-      <c r="J40" s="73"/>
-      <c r="K40" s="73"/>
-      <c r="L40" s="73"/>
+      <c r="H40" s="71"/>
+      <c r="I40" s="71"/>
+      <c r="J40" s="71"/>
+      <c r="K40" s="71"/>
+      <c r="L40" s="71"/>
     </row>
     <row r="41" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A41" s="46" t="s">
@@ -7926,11 +7994,11 @@
         <f>E40</f>
         <v>Total</v>
       </c>
-      <c r="H52" s="73"/>
-      <c r="I52" s="73"/>
-      <c r="J52" s="73"/>
-      <c r="K52" s="73"/>
-      <c r="L52" s="73"/>
+      <c r="H52" s="71"/>
+      <c r="I52" s="71"/>
+      <c r="J52" s="71"/>
+      <c r="K52" s="71"/>
+      <c r="L52" s="71"/>
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A53" s="50" t="str">
@@ -8188,11 +8256,11 @@
         <f>SUM(E41:E42)/$E$49</f>
         <v>0.47599999999999992</v>
       </c>
-      <c r="H64" s="73"/>
-      <c r="I64" s="73"/>
-      <c r="J64" s="73"/>
-      <c r="K64" s="73"/>
-      <c r="L64" s="73"/>
+      <c r="H64" s="71"/>
+      <c r="I64" s="71"/>
+      <c r="J64" s="71"/>
+      <c r="K64" s="71"/>
+      <c r="L64" s="71"/>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A65" s="48" t="s">
@@ -8330,12 +8398,17 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="H52:L52"/>
-    <mergeCell ref="H64:L64"/>
-    <mergeCell ref="H40:L40"/>
-    <mergeCell ref="D34:D36"/>
-    <mergeCell ref="E34:E36"/>
-    <mergeCell ref="F34:F36"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="B34:B36"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="C32:C33"/>
+    <mergeCell ref="C34:C36"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="H2:L2"/>
+    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="H14:L14"/>
+    <mergeCell ref="A27:E27"/>
     <mergeCell ref="E32:E33"/>
     <mergeCell ref="H27:L27"/>
     <mergeCell ref="F29:F30"/>
@@ -8343,17 +8416,12 @@
     <mergeCell ref="D29:D30"/>
     <mergeCell ref="D32:D33"/>
     <mergeCell ref="E29:E30"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="H2:L2"/>
-    <mergeCell ref="A14:E14"/>
-    <mergeCell ref="H14:L14"/>
-    <mergeCell ref="A27:E27"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="B34:B36"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="C32:C33"/>
-    <mergeCell ref="C34:C36"/>
+    <mergeCell ref="H52:L52"/>
+    <mergeCell ref="H64:L64"/>
+    <mergeCell ref="H40:L40"/>
+    <mergeCell ref="D34:D36"/>
+    <mergeCell ref="E34:E36"/>
+    <mergeCell ref="F34:F36"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Calibration Pipeline Script Update
Minor adjustment in excel formula in CDAP template
</commit_message>
<xml_diff>
--- a/utilities/calibration/workbook_templates/04_CoordinatedDailyActivityPattern_2023_blank.xlsx
+++ b/utilities/calibration/workbook_templates/04_CoordinatedDailyActivityPattern_2023_blank.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub\travel-model-one-tm1.7_calibration\utilities\calibration\workbook_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D06DF58-9916-4B5E-A7BD-6A25D6896A95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1330CBA-E079-4F3E-9BDD-2031FF7E0A01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="calibration" sheetId="1" r:id="rId1"/>
@@ -32,8 +32,8 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="40" r:id="rId8"/>
-    <pivotCache cacheId="41" r:id="rId9"/>
+    <pivotCache cacheId="66" r:id="rId8"/>
+    <pivotCache cacheId="67" r:id="rId9"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -808,13 +808,13 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="8" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="3" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="5" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2802,7 +2802,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{EC85B2BF-B5A3-41FF-B478-F9EFC1F3C73E}" name="PivotTable1" cacheId="40" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{EC85B2BF-B5A3-41FF-B478-F9EFC1F3C73E}" name="PivotTable1" cacheId="66" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="P4:AB16" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField axis="axisRow" showAll="0">
@@ -2935,7 +2935,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FD0500BC-8277-4543-8FF3-B18D1357F7D3}" name="PivotTable5" cacheId="41" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FD0500BC-8277-4543-8FF3-B18D1357F7D3}" name="PivotTable5" cacheId="67" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="I5:M15" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField axis="axisRow" showAll="0">
@@ -5661,6 +5661,10 @@
         <f t="shared" si="46"/>
         <v>8</v>
       </c>
+      <c r="Q54" s="5">
+        <f>SUM(Q46:Q53)</f>
+        <v>48</v>
+      </c>
       <c r="S54" s="5">
         <f>IFERROR(K54-C54,0)</f>
         <v>-2935344.4913071152</v>
@@ -6552,52 +6556,52 @@
         <v>1</v>
       </c>
       <c r="K67" s="17">
-        <f>IFERROR(K54/$N54,0)</f>
-        <v>1</v>
+        <f>IFERROR(K54/$Q54,0)</f>
+        <v>0.16666666666666666</v>
       </c>
       <c r="L67" s="17">
-        <f>IFERROR(L54/$N54,0)</f>
-        <v>1</v>
+        <f t="shared" ref="L67:P67" si="72">IFERROR(L54/$Q54,0)</f>
+        <v>0.16666666666666666</v>
       </c>
       <c r="M67" s="17">
-        <f>IFERROR(M54/$N54,0)</f>
-        <v>1</v>
+        <f t="shared" si="72"/>
+        <v>0.16666666666666666</v>
       </c>
       <c r="N67" s="17">
-        <f>IFERROR(N54/$N54,0)</f>
-        <v>1</v>
+        <f t="shared" si="72"/>
+        <v>0.16666666666666666</v>
       </c>
       <c r="O67" s="17">
-        <f t="shared" ref="O67:P67" si="72">IFERROR(O54/$N54,0)</f>
-        <v>1</v>
+        <f t="shared" si="72"/>
+        <v>0.16666666666666666</v>
       </c>
       <c r="P67" s="17">
         <f t="shared" si="72"/>
-        <v>1</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="S67" s="17">
         <f t="shared" si="51"/>
-        <v>0.60165995276335349</v>
+        <v>-0.23167338056997991</v>
       </c>
       <c r="T67" s="17">
         <f t="shared" si="52"/>
-        <v>0.99899794940008879</v>
+        <v>0.16566461606675542</v>
       </c>
       <c r="U67" s="17">
         <f t="shared" si="53"/>
-        <v>0.71234611843767126</v>
+        <v>-0.12098721489566208</v>
       </c>
       <c r="V67" s="17">
         <f t="shared" si="54"/>
-        <v>0.87357856116241783</v>
+        <v>4.0245227829084462E-2</v>
       </c>
       <c r="W67" s="17">
         <f t="shared" si="54"/>
-        <v>0.86571367460189408</v>
+        <v>3.2380341268560792E-2</v>
       </c>
       <c r="X67" s="17">
         <f t="shared" si="54"/>
-        <v>0.94770374363457455</v>
+        <v>0.11437041030124116</v>
       </c>
     </row>
   </sheetData>
@@ -9330,19 +9334,19 @@
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" s="97" t="s">
+      <c r="A2" s="96" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="97"/>
-      <c r="C2" s="97"/>
-      <c r="D2" s="97"/>
-      <c r="E2" s="97"/>
+      <c r="B2" s="96"/>
+      <c r="C2" s="96"/>
+      <c r="D2" s="96"/>
+      <c r="E2" s="96"/>
       <c r="F2" s="60"/>
-      <c r="H2" s="95"/>
-      <c r="I2" s="95"/>
-      <c r="J2" s="95"/>
-      <c r="K2" s="95"/>
-      <c r="L2" s="95"/>
+      <c r="H2" s="97"/>
+      <c r="I2" s="97"/>
+      <c r="J2" s="97"/>
+      <c r="K2" s="97"/>
+      <c r="L2" s="97"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="50" t="s">
@@ -9611,19 +9615,19 @@
       <c r="F13" s="50"/>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A14" s="97" t="s">
+      <c r="A14" s="96" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="97"/>
-      <c r="C14" s="97"/>
-      <c r="D14" s="97"/>
-      <c r="E14" s="97"/>
+      <c r="B14" s="96"/>
+      <c r="C14" s="96"/>
+      <c r="D14" s="96"/>
+      <c r="E14" s="96"/>
       <c r="F14" s="60"/>
-      <c r="H14" s="95"/>
-      <c r="I14" s="95"/>
-      <c r="J14" s="95"/>
-      <c r="K14" s="95"/>
-      <c r="L14" s="95"/>
+      <c r="H14" s="97"/>
+      <c r="I14" s="97"/>
+      <c r="J14" s="97"/>
+      <c r="K14" s="97"/>
+      <c r="L14" s="97"/>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="50" t="s">
@@ -9885,19 +9889,19 @@
       <c r="A25" s="57"/>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A27" s="95" t="s">
+      <c r="A27" s="97" t="s">
         <v>32</v>
       </c>
-      <c r="B27" s="95"/>
-      <c r="C27" s="95"/>
-      <c r="D27" s="95"/>
-      <c r="E27" s="95"/>
+      <c r="B27" s="97"/>
+      <c r="C27" s="97"/>
+      <c r="D27" s="97"/>
+      <c r="E27" s="97"/>
       <c r="F27" s="56"/>
-      <c r="H27" s="95"/>
-      <c r="I27" s="95"/>
-      <c r="J27" s="95"/>
-      <c r="K27" s="95"/>
-      <c r="L27" s="95"/>
+      <c r="H27" s="97"/>
+      <c r="I27" s="97"/>
+      <c r="J27" s="97"/>
+      <c r="K27" s="97"/>
+      <c r="L27" s="97"/>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="46" t="s">
@@ -9927,20 +9931,20 @@
       <c r="A29" s="46" t="s">
         <v>6</v>
       </c>
-      <c r="B29" s="96">
+      <c r="B29" s="95">
         <v>0.79</v>
       </c>
-      <c r="C29" s="96">
+      <c r="C29" s="95">
         <v>0.12</v>
       </c>
-      <c r="D29" s="96">
+      <c r="D29" s="95">
         <v>0.09</v>
       </c>
-      <c r="E29" s="96">
+      <c r="E29" s="95">
         <f>SUM(B29:D29)</f>
         <v>1</v>
       </c>
-      <c r="F29" s="96">
+      <c r="F29" s="95">
         <v>0.47599999999999998</v>
       </c>
       <c r="I29" s="64"/>
@@ -9952,11 +9956,11 @@
       <c r="A30" s="46" t="s">
         <v>7</v>
       </c>
-      <c r="B30" s="96"/>
-      <c r="C30" s="96"/>
-      <c r="D30" s="96"/>
-      <c r="E30" s="96"/>
-      <c r="F30" s="96"/>
+      <c r="B30" s="95"/>
+      <c r="C30" s="95"/>
+      <c r="D30" s="95"/>
+      <c r="E30" s="95"/>
+      <c r="F30" s="95"/>
       <c r="I30" s="64"/>
       <c r="J30" s="64"/>
       <c r="K30" s="64"/>
@@ -9991,20 +9995,20 @@
       <c r="A32" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="B32" s="96">
-        <v>0</v>
-      </c>
-      <c r="C32" s="96">
+      <c r="B32" s="95">
+        <v>0</v>
+      </c>
+      <c r="C32" s="95">
         <v>0.8</v>
       </c>
-      <c r="D32" s="96">
+      <c r="D32" s="95">
         <v>0.2</v>
       </c>
-      <c r="E32" s="96">
+      <c r="E32" s="95">
         <f>SUM(B32:D32)</f>
         <v>1</v>
       </c>
-      <c r="F32" s="96">
+      <c r="F32" s="95">
         <v>0.22600000000000001</v>
       </c>
       <c r="I32" s="64"/>
@@ -10016,11 +10020,11 @@
       <c r="A33" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="B33" s="96"/>
-      <c r="C33" s="96"/>
-      <c r="D33" s="96"/>
-      <c r="E33" s="96"/>
-      <c r="F33" s="96"/>
+      <c r="B33" s="95"/>
+      <c r="C33" s="95"/>
+      <c r="D33" s="95"/>
+      <c r="E33" s="95"/>
+      <c r="F33" s="95"/>
       <c r="I33" s="64"/>
       <c r="J33" s="64"/>
       <c r="K33" s="64"/>
@@ -10030,20 +10034,20 @@
       <c r="A34" s="46" t="s">
         <v>11</v>
       </c>
-      <c r="B34" s="96">
+      <c r="B34" s="95">
         <v>0.65</v>
       </c>
-      <c r="C34" s="96">
+      <c r="C34" s="95">
         <v>0.2</v>
       </c>
-      <c r="D34" s="96">
+      <c r="D34" s="95">
         <v>0.15</v>
       </c>
-      <c r="E34" s="96">
+      <c r="E34" s="95">
         <f>SUM(B34:D34)</f>
         <v>1</v>
       </c>
-      <c r="F34" s="96">
+      <c r="F34" s="95">
         <v>0.246</v>
       </c>
       <c r="I34" s="64"/>
@@ -10055,11 +10059,11 @@
       <c r="A35" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="B35" s="96"/>
-      <c r="C35" s="96"/>
-      <c r="D35" s="96"/>
-      <c r="E35" s="96"/>
-      <c r="F35" s="96"/>
+      <c r="B35" s="95"/>
+      <c r="C35" s="95"/>
+      <c r="D35" s="95"/>
+      <c r="E35" s="95"/>
+      <c r="F35" s="95"/>
       <c r="I35" s="64"/>
       <c r="J35" s="64"/>
       <c r="K35" s="64"/>
@@ -10069,11 +10073,11 @@
       <c r="A36" s="46" t="s">
         <v>13</v>
       </c>
-      <c r="B36" s="96"/>
-      <c r="C36" s="96"/>
-      <c r="D36" s="96"/>
-      <c r="E36" s="96"/>
-      <c r="F36" s="96"/>
+      <c r="B36" s="95"/>
+      <c r="C36" s="95"/>
+      <c r="D36" s="95"/>
+      <c r="E36" s="95"/>
+      <c r="F36" s="95"/>
       <c r="I36" s="64"/>
       <c r="J36" s="64"/>
       <c r="K36" s="64"/>
@@ -10133,11 +10137,11 @@
       <c r="F40" s="54" t="s">
         <v>31</v>
       </c>
-      <c r="H40" s="95"/>
-      <c r="I40" s="95"/>
-      <c r="J40" s="95"/>
-      <c r="K40" s="95"/>
-      <c r="L40" s="95"/>
+      <c r="H40" s="97"/>
+      <c r="I40" s="97"/>
+      <c r="J40" s="97"/>
+      <c r="K40" s="97"/>
+      <c r="L40" s="97"/>
     </row>
     <row r="41" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A41" s="46" t="s">
@@ -10425,11 +10429,11 @@
         <f>E40</f>
         <v>Total</v>
       </c>
-      <c r="H52" s="95"/>
-      <c r="I52" s="95"/>
-      <c r="J52" s="95"/>
-      <c r="K52" s="95"/>
-      <c r="L52" s="95"/>
+      <c r="H52" s="97"/>
+      <c r="I52" s="97"/>
+      <c r="J52" s="97"/>
+      <c r="K52" s="97"/>
+      <c r="L52" s="97"/>
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A53" s="50" t="str">
@@ -10687,11 +10691,11 @@
         <f>SUM(E41:E42)/$E$49</f>
         <v>0.47599999999999992</v>
       </c>
-      <c r="H64" s="95"/>
-      <c r="I64" s="95"/>
-      <c r="J64" s="95"/>
-      <c r="K64" s="95"/>
-      <c r="L64" s="95"/>
+      <c r="H64" s="97"/>
+      <c r="I64" s="97"/>
+      <c r="J64" s="97"/>
+      <c r="K64" s="97"/>
+      <c r="L64" s="97"/>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A65" s="48" t="s">
@@ -10829,17 +10833,12 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="B34:B36"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="C32:C33"/>
-    <mergeCell ref="C34:C36"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="H2:L2"/>
-    <mergeCell ref="A14:E14"/>
-    <mergeCell ref="H14:L14"/>
-    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="H52:L52"/>
+    <mergeCell ref="H64:L64"/>
+    <mergeCell ref="H40:L40"/>
+    <mergeCell ref="D34:D36"/>
+    <mergeCell ref="E34:E36"/>
+    <mergeCell ref="F34:F36"/>
     <mergeCell ref="E32:E33"/>
     <mergeCell ref="H27:L27"/>
     <mergeCell ref="F29:F30"/>
@@ -10847,12 +10846,17 @@
     <mergeCell ref="D29:D30"/>
     <mergeCell ref="D32:D33"/>
     <mergeCell ref="E29:E30"/>
-    <mergeCell ref="H52:L52"/>
-    <mergeCell ref="H64:L64"/>
-    <mergeCell ref="H40:L40"/>
-    <mergeCell ref="D34:D36"/>
-    <mergeCell ref="E34:E36"/>
-    <mergeCell ref="F34:F36"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="H2:L2"/>
+    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="H14:L14"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="B34:B36"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="C32:C33"/>
+    <mergeCell ref="C34:C36"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>